<commit_message>
fix: regenerate Scenarios.xlsx without Facts sheet
- Removed Facts sheet from example Excel file
- File now only contains Scenarios sheet with 100 entries
- Matches current codebase after facts feature removal
</commit_message>
<xml_diff>
--- a/public/assets/Scenarios.xlsx
+++ b/public/assets/Scenarios.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="Scenarios" sheetId="1" r:id="rId4"/>
-    <sheet name="Facts" sheetId="2" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
@@ -16,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="262">
   <si>
     <t>StrtNm</t>
   </si>
@@ -802,69 +801,6 @@
   </si>
   <si>
     <t>Bâtiment Est</t>
-  </si>
-  <si>
-    <t>Fact</t>
-  </si>
-  <si>
-    <t>ISO 20022 is used by over 200 market infrastructures across 70+ countries worldwide.</t>
-  </si>
-  <si>
-    <t>The SWIFT network processes an average of 44.8 million messages per day.</t>
-  </si>
-  <si>
-    <t>Structured addresses reduce payment repair rates by up to 40%.</t>
-  </si>
-  <si>
-    <t>ISO 20022 supports 10 address components, replacing the legacy 4-line free-text format.</t>
-  </si>
-  <si>
-    <t>The &lt;TwnNm&gt; and &lt;Ctry&gt; fields are the only mandatory address elements in ISO 20022.</t>
-  </si>
-  <si>
-    <t>Country codes in ISO 20022 must follow the ISO 3166-1 alpha-2 standard (2-letter codes).</t>
-  </si>
-  <si>
-    <t>Each &lt;AdrLine&gt; element in hybrid mode is limited to 70 characters maximum.</t>
-  </si>
-  <si>
-    <t>SWIFT's CBPR+ guidelines require structured addresses for cross-border payments from 2026.</t>
-  </si>
-  <si>
-    <t>The European Payments Council mandates ISO 20022 for all SEPA transactions.</t>
-  </si>
-  <si>
-    <t>ISO 20022 was first published in 2004 and has been adopted globally over two decades.</t>
-  </si>
-  <si>
-    <t>Hybrid addressing allows mixing structured fields with free-text address lines.</t>
-  </si>
-  <si>
-    <t>The &lt;BldgNb&gt; field can contain letters and numbers (e.g., "221B").</t>
-  </si>
-  <si>
-    <t>ISO 20022 address data improves sanctions screening accuracy by 25%.</t>
-  </si>
-  <si>
-    <t>The Fedwire Funds Service migrated to ISO 20022 in March 2025.</t>
-  </si>
-  <si>
-    <t>Over 10,000 financial institutions worldwide exchange ISO 20022 messages daily.</t>
-  </si>
-  <si>
-    <t>The Bank of England adopted ISO 20022 for CHAPS in June 2023.</t>
-  </si>
-  <si>
-    <t>Structured addresses enable straight-through processing (STP) without manual intervention.</t>
-  </si>
-  <si>
-    <t>In ISO 20022, &lt;PstCd&gt; (Postal Code) is optional but strongly recommended for accuracy.</t>
-  </si>
-  <si>
-    <t>The TARGET2 system in the Eurozone completed its migration to ISO 20022 in March 2023.</t>
-  </si>
-  <si>
-    <t>ISO 20022 messages use XML syntax and can represent over 400 different business processes.</t>
   </si>
 </sst>
 </file>
@@ -3459,136 +3395,4 @@
   </headerFooter>
   <tableParts count="0"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:A21"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col min="1" max="1" width="107.26" bestFit="true" customWidth="true" style="0"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1">
-      <c r="A2" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1">
-      <c r="A3" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1">
-      <c r="A4" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1">
-      <c r="A5" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1">
-      <c r="A6" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1">
-      <c r="A7" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1">
-      <c r="A8" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1">
-      <c r="A9" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1">
-      <c r="A10" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1">
-      <c r="A11" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1">
-      <c r="A12" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1">
-      <c r="A13" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1">
-      <c r="A14" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1">
-      <c r="A15" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1">
-      <c r="A16" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1">
-      <c r="A17" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1">
-      <c r="A18" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1">
-      <c r="A19" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1">
-      <c r="A20" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1">
-      <c r="A21" t="s">
-        <v>282</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions gridLines="false" gridLinesSet="true"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
-  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddHeader/>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-  <tableParts count="0"/>
-</worksheet>
 </file>
</xml_diff>